<commit_message>
versión calculo de kilometros 11/03
</commit_message>
<xml_diff>
--- a/public/data/matriz-distancias.xlsx
+++ b/public/data/matriz-distancias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://descargasjosan.sharepoint.com/sites/ArchivosDescargasJosan/Documentos compartidos/AGENDA/Aplicación/App Nueva/public/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{2F953D46-F199-46EB-8D65-37B6D13238A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F38801D4-3DA6-48D9-83EB-D8BDD3B2A2A6}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{2F953D46-F199-46EB-8D65-37B6D13238A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6B55F2D-6470-4DED-8A26-A0855D8926D3}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D0FB8F1A-4061-47AE-9F43-39E496646E02}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="38">
   <si>
     <t>ARTE REGAL IMPORT, S.L. - MANISES</t>
   </si>
@@ -147,6 +147,9 @@
   </si>
   <si>
     <t>OFICINA - VALENCIA</t>
+  </si>
+  <si>
+    <t>AMERICOLD VALENCIA SL UNIPERSONAL - VALENCIA</t>
   </si>
 </sst>
 </file>
@@ -518,7 +521,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBE320F9-4947-4ED6-B94D-306C2D1C4CA5}">
-  <dimension ref="A1:AL38"/>
+  <dimension ref="A1:AM39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="54.109375" bestFit="1" customWidth="1"/>
@@ -559,9 +562,10 @@
     <col min="36" max="36" width="25.44140625" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="33.77734375" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="44.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:39" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -673,8 +677,11 @@
       <c r="AL1" t="s">
         <v>36</v>
       </c>
+      <c r="AM1" t="s">
+        <v>37</v>
+      </c>
     </row>
-    <row r="2" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -789,8 +796,11 @@
       <c r="AL2">
         <v>10.210000000000001</v>
       </c>
+      <c r="AM2">
+        <v>16.690000000000001</v>
+      </c>
     </row>
-    <row r="3" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -905,8 +915,11 @@
       <c r="AL3">
         <v>14.05</v>
       </c>
+      <c r="AM3">
+        <v>20.61</v>
+      </c>
     </row>
-    <row r="4" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1021,8 +1034,11 @@
       <c r="AL4">
         <v>20.47</v>
       </c>
+      <c r="AM4">
+        <v>26.93</v>
+      </c>
     </row>
-    <row r="5" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1137,8 +1153,11 @@
       <c r="AL5">
         <v>8.25</v>
       </c>
+      <c r="AM5">
+        <v>14.26</v>
+      </c>
     </row>
-    <row r="6" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1250,8 +1269,11 @@
       <c r="AL6">
         <v>12.03</v>
       </c>
+      <c r="AM6">
+        <v>18.579999999999998</v>
+      </c>
     </row>
-    <row r="7" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1366,8 +1388,11 @@
       <c r="AL7">
         <v>26.64</v>
       </c>
+      <c r="AM7">
+        <v>26.38</v>
+      </c>
     </row>
-    <row r="8" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1476,8 +1501,11 @@
       <c r="AL8">
         <v>8.5399999999999991</v>
       </c>
+      <c r="AM8">
+        <v>14.63</v>
+      </c>
     </row>
-    <row r="9" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1589,8 +1617,11 @@
       <c r="AL9">
         <v>45.78</v>
       </c>
+      <c r="AM9">
+        <v>46.13</v>
+      </c>
     </row>
-    <row r="10" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1705,8 +1736,11 @@
       <c r="AL10">
         <v>8.75</v>
       </c>
+      <c r="AM10">
+        <v>14.51</v>
+      </c>
     </row>
-    <row r="11" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1821,8 +1855,11 @@
       <c r="AL11">
         <v>12.15</v>
       </c>
+      <c r="AM11">
+        <v>18.670000000000002</v>
+      </c>
     </row>
-    <row r="12" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1937,8 +1974,11 @@
       <c r="AL12">
         <v>16.72</v>
       </c>
+      <c r="AM12">
+        <v>16.079999999999998</v>
+      </c>
     </row>
-    <row r="13" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -2053,8 +2093,11 @@
       <c r="AL13">
         <v>13.94</v>
       </c>
+      <c r="AM13">
+        <v>15.05</v>
+      </c>
     </row>
-    <row r="14" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -2169,8 +2212,11 @@
       <c r="AL14">
         <v>20.16</v>
       </c>
+      <c r="AM14">
+        <v>20.3</v>
+      </c>
     </row>
-    <row r="15" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -2285,8 +2331,11 @@
       <c r="AL15">
         <v>15.39</v>
       </c>
+      <c r="AM15">
+        <v>18.34</v>
+      </c>
     </row>
-    <row r="16" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -2401,8 +2450,11 @@
       <c r="AL16">
         <v>14.1</v>
       </c>
+      <c r="AM16">
+        <v>20.64</v>
+      </c>
     </row>
-    <row r="17" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -2517,8 +2569,11 @@
       <c r="AL17">
         <v>14.52</v>
       </c>
+      <c r="AM17">
+        <v>21.05</v>
+      </c>
     </row>
-    <row r="18" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -2630,8 +2685,11 @@
       <c r="AL18">
         <v>3.03</v>
       </c>
+      <c r="AM18">
+        <v>6.76</v>
+      </c>
     </row>
-    <row r="19" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -2746,8 +2804,11 @@
       <c r="AL19">
         <v>11.48</v>
       </c>
+      <c r="AM19">
+        <v>18.059999999999999</v>
+      </c>
     </row>
-    <row r="20" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -2859,8 +2920,11 @@
       <c r="AL20">
         <v>58.6</v>
       </c>
+      <c r="AM20">
+        <v>58.61</v>
+      </c>
     </row>
-    <row r="21" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -2972,8 +3036,11 @@
       <c r="AL21">
         <v>63.99</v>
       </c>
+      <c r="AM21">
+        <v>63.14</v>
+      </c>
     </row>
-    <row r="22" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -3088,8 +3155,11 @@
       <c r="AL22">
         <v>15.35</v>
       </c>
+      <c r="AM22">
+        <v>21.85</v>
+      </c>
     </row>
-    <row r="23" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -3204,8 +3274,11 @@
       <c r="AL23">
         <v>6.06</v>
       </c>
+      <c r="AM23">
+        <v>2.08</v>
+      </c>
     </row>
-    <row r="24" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -3320,8 +3393,11 @@
       <c r="AL24">
         <v>13.63</v>
       </c>
+      <c r="AM24">
+        <v>20.13</v>
+      </c>
     </row>
-    <row r="25" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -3436,8 +3512,11 @@
       <c r="AL25">
         <v>15.94</v>
       </c>
+      <c r="AM25">
+        <v>22.47</v>
+      </c>
     </row>
-    <row r="26" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>24</v>
       </c>
@@ -3552,8 +3631,11 @@
       <c r="AL26">
         <v>13.63</v>
       </c>
+      <c r="AM26">
+        <v>20.13</v>
+      </c>
     </row>
-    <row r="27" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -3668,8 +3750,11 @@
       <c r="AL27">
         <v>14</v>
       </c>
+      <c r="AM27">
+        <v>20.54</v>
+      </c>
     </row>
-    <row r="28" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -3781,8 +3866,11 @@
       <c r="AL28">
         <v>7.92</v>
       </c>
+      <c r="AM28">
+        <v>14.48</v>
+      </c>
     </row>
-    <row r="29" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -3897,8 +3985,11 @@
       <c r="AL29">
         <v>15.61</v>
       </c>
+      <c r="AM29">
+        <v>22.1</v>
+      </c>
     </row>
-    <row r="30" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -4013,8 +4104,11 @@
       <c r="AL30">
         <v>15.15</v>
       </c>
+      <c r="AM30">
+        <v>15.61</v>
+      </c>
     </row>
-    <row r="31" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>29</v>
       </c>
@@ -4129,8 +4223,11 @@
       <c r="AL31">
         <v>8.01</v>
       </c>
+      <c r="AM31">
+        <v>14.54</v>
+      </c>
     </row>
-    <row r="32" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>30</v>
       </c>
@@ -4245,8 +4342,11 @@
       <c r="AL32">
         <v>11.7</v>
       </c>
+      <c r="AM32">
+        <v>18.28</v>
+      </c>
     </row>
-    <row r="33" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>31</v>
       </c>
@@ -4361,8 +4461,11 @@
       <c r="AL33">
         <v>26.03</v>
       </c>
+      <c r="AM33">
+        <v>25.61</v>
+      </c>
     </row>
-    <row r="34" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>32</v>
       </c>
@@ -4477,8 +4580,11 @@
       <c r="AL34">
         <v>15.35</v>
       </c>
+      <c r="AM34">
+        <v>21.86</v>
+      </c>
     </row>
-    <row r="35" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>33</v>
       </c>
@@ -4593,8 +4699,11 @@
       <c r="AL35">
         <v>11.98</v>
       </c>
+      <c r="AM35">
+        <v>15.36</v>
+      </c>
     </row>
-    <row r="36" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>34</v>
       </c>
@@ -4709,8 +4818,11 @@
       <c r="AL36">
         <v>12.34</v>
       </c>
+      <c r="AM36">
+        <v>11.39</v>
+      </c>
     </row>
-    <row r="37" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>35</v>
       </c>
@@ -4825,8 +4937,11 @@
       <c r="AL37">
         <v>12.49</v>
       </c>
+      <c r="AM37">
+        <v>12.89</v>
+      </c>
     </row>
-    <row r="38" spans="1:38" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>36</v>
       </c>
@@ -4939,6 +5054,128 @@
         <v>12.49</v>
       </c>
       <c r="AL38">
+        <v>0</v>
+      </c>
+      <c r="AM38">
+        <v>6.57</v>
+      </c>
+    </row>
+    <row r="39" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>37</v>
+      </c>
+      <c r="B39">
+        <v>16.690000000000001</v>
+      </c>
+      <c r="C39">
+        <v>20.61</v>
+      </c>
+      <c r="D39">
+        <v>26.93</v>
+      </c>
+      <c r="E39">
+        <v>14.26</v>
+      </c>
+      <c r="F39">
+        <v>18.579999999999998</v>
+      </c>
+      <c r="G39">
+        <v>26.38</v>
+      </c>
+      <c r="H39">
+        <v>14.63</v>
+      </c>
+      <c r="I39">
+        <v>46.13</v>
+      </c>
+      <c r="J39">
+        <v>14.51</v>
+      </c>
+      <c r="K39">
+        <v>18.670000000000002</v>
+      </c>
+      <c r="L39">
+        <v>16.079999999999998</v>
+      </c>
+      <c r="M39">
+        <v>15.05</v>
+      </c>
+      <c r="N39">
+        <v>20.3</v>
+      </c>
+      <c r="O39">
+        <v>18.34</v>
+      </c>
+      <c r="P39">
+        <v>20.64</v>
+      </c>
+      <c r="Q39">
+        <v>21.05</v>
+      </c>
+      <c r="R39">
+        <v>6.76</v>
+      </c>
+      <c r="S39">
+        <v>18.059999999999999</v>
+      </c>
+      <c r="T39">
+        <v>58.61</v>
+      </c>
+      <c r="U39">
+        <v>63.14</v>
+      </c>
+      <c r="V39">
+        <v>21.85</v>
+      </c>
+      <c r="W39">
+        <v>2.08</v>
+      </c>
+      <c r="X39">
+        <v>20.13</v>
+      </c>
+      <c r="Y39">
+        <v>22.47</v>
+      </c>
+      <c r="Z39">
+        <v>20.13</v>
+      </c>
+      <c r="AA39">
+        <v>20.54</v>
+      </c>
+      <c r="AB39">
+        <v>14.48</v>
+      </c>
+      <c r="AC39">
+        <v>22.1</v>
+      </c>
+      <c r="AD39">
+        <v>15.61</v>
+      </c>
+      <c r="AE39">
+        <v>14.54</v>
+      </c>
+      <c r="AF39">
+        <v>18.28</v>
+      </c>
+      <c r="AG39">
+        <v>25.61</v>
+      </c>
+      <c r="AH39">
+        <v>21.86</v>
+      </c>
+      <c r="AI39">
+        <v>15.36</v>
+      </c>
+      <c r="AJ39">
+        <v>11.39</v>
+      </c>
+      <c r="AK39">
+        <v>12.89</v>
+      </c>
+      <c r="AL39">
+        <v>6.57</v>
+      </c>
+      <c r="AM39">
         <v>0</v>
       </c>
     </row>
@@ -4948,17 +5185,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="997f4d01-1611-4e90-8cef-12d6214bbbe2">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="f8d013da-fb2b-48a4-87bf-4b65d2faa275" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010037B70B819506B8459DDD68EE2BB294CC" ma:contentTypeVersion="11" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="45c6a4bbc3a3039899d05f93d6b397b0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="997f4d01-1611-4e90-8cef-12d6214bbbe2" xmlns:ns3="f8d013da-fb2b-48a4-87bf-4b65d2faa275" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5b10260ac49b06150e809f313ea727a8" ns2:_="" ns3:_="">
     <xsd:import namespace="997f4d01-1611-4e90-8cef-12d6214bbbe2"/>
@@ -5153,6 +5379,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="997f4d01-1611-4e90-8cef-12d6214bbbe2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="f8d013da-fb2b-48a4-87bf-4b65d2faa275" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -5163,17 +5400,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1E7247F-EF4A-47C2-8CCB-8692A6AA65E4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="997f4d01-1611-4e90-8cef-12d6214bbbe2"/>
-    <ds:schemaRef ds:uri="f8d013da-fb2b-48a4-87bf-4b65d2faa275"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0B18FFA1-1D92-49D8-8985-C20147E1AF3B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5192,6 +5418,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1E7247F-EF4A-47C2-8CCB-8692A6AA65E4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="997f4d01-1611-4e90-8cef-12d6214bbbe2"/>
+    <ds:schemaRef ds:uri="f8d013da-fb2b-48a4-87bf-4b65d2faa275"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5D31D42-3C5D-4787-BD23-B13ED7F270D1}">
   <ds:schemaRefs>

</xml_diff>